<commit_message>
CS0073 M2: make Full workbook stand alone for the group's Excel submission
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Statistical Analysis and Modeling/PAMESA - M2-Technical - Full.xlsx
+++ b/Statistical Analysis and Modeling/PAMESA - M2-Technical - Full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\School-Works\Statistical Analysis and Modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DBFCFA-AAEA-47AE-950F-D73D91DD20BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B982E435-37DB-47D6-A81D-ED702C7823BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="250">
   <si>
     <t>CS0073 Technical Assessment, Module 2: Diagnostic Analytics and Statistical Inference</t>
   </si>
@@ -82,12 +82,6 @@
   </si>
   <si>
     <t>Customer_Satisfaction.xlsx: restaurant survey, 405 respondents, 13 items on a 1 to 7 scale</t>
-  </si>
-  <si>
-    <t>Companion file</t>
-  </si>
-  <si>
-    <t>PAMESA - M2-Technical - Full.ipynb (same analysis in Python, plus Tukey post-hoc, Shapiro-Wilk and Spearman, which Excel cannot compute directly)</t>
   </si>
   <si>
     <t>Sheets, in order</t>
@@ -480,9 +474,6 @@
     <t>Strength labels (rule of thumb): below 0.10 negligible, 0.10 to 0.29 weak, 0.30 to 0.49 moderate, 0.50 to 0.69 strong, 0.70 and up very strong.</t>
   </si>
   <si>
-    <t>Spearman (rank) correlations, a robustness check, are in the notebook; they never differ from Pearson by more than 0.07.</t>
-  </si>
-  <si>
     <t>x15 freshness (group)</t>
   </si>
   <si>
@@ -627,9 +618,6 @@
     <t>df2</t>
   </si>
   <si>
-    <t>Excel's F.DIST.RT rounds df2 down to a whole number (176), so this p differs from Python's in the far decimal places; the decision is the same.</t>
-  </si>
-  <si>
     <t>Remedy 2. Kruskal-Wallis test (compares ranks; no normality or equal-variance assumption)</t>
   </si>
   <si>
@@ -667,9 +655,6 @@
   </si>
   <si>
     <t>Kruskal-Wallis (H)</t>
-  </si>
-  <si>
-    <t>Post-hoc (which pairs differ): Tukey's HSD is in the notebook, because Excel has no studentized range function. Normality (Shapiro-Wilk) is also tested in the notebook.</t>
   </si>
   <si>
     <t>Perception (sorted)</t>
@@ -793,6 +778,24 @@
   </si>
   <si>
     <t>Correction 3: after the assumption checks failed, Welch's ANOVA and Kruskal-Wallis were added; the conclusion rests on all three tests agreeing.</t>
+  </si>
+  <si>
+    <t>Scope note</t>
+  </si>
+  <si>
+    <t>Tukey's HSD post-hoc test and the Shapiro-Wilk normality test are not included because Excel has no built-in functions for them. Welch's ANOVA and Kruskal-Wallis are included instead as checks that do not rely on equal variances or normality.</t>
+  </si>
+  <si>
+    <t>Pearson r is used throughout this sheet.</t>
+  </si>
+  <si>
+    <t>Excel's F.DIST.RT rounds df2 down to a whole number (176), so this p-value is approximate in the far decimal places; the decision is the same.</t>
+  </si>
+  <si>
+    <t>Post-hoc (which pairs differ): Tukey's HSD is not included because Excel has no studentized range function. The group means rise at every freshness level (3.99, 4.35, 4.85, 5.51), as the chart on the Charts sheet shows.</t>
+  </si>
+  <si>
+    <t>Submission format: the group submits in Excel, so this workbook is the deliverable. The Python notebook was used only to cross-check the values above.</t>
   </si>
 </sst>
 </file>
@@ -1749,124 +1752,124 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>244</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1886,162 +1889,162 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B4" s="28" t="str">
         <f>Cleaning!B4&amp;" / "&amp;Cleaning!B5&amp;" / "&amp;Cleaning!B6&amp;" / "&amp;Cleaning!B7</f>
         <v>405 / 0 / 0 / 0</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B5" s="30">
         <f>Correlation!B7</f>
         <v>9.746066407377954E-2</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B6" s="30">
         <f>Correlation!C29</f>
         <v>0.55855337039537545</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B7" s="31">
         <f>Correlation!C37</f>
         <v>30</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B8" s="28" t="str">
         <f>TEXT(ANOVA!B21,"0.00")&amp;" (p = "&amp;TEXT(ANOVA!B22,"0.0E+00")&amp;")"</f>
         <v>38.60 (p = 6.2E-22)</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B9" s="28" t="str">
         <f>TEXT(ANOVA!E27,"0.00")&amp;"  (df = "&amp;ANOVA!C27&amp;", "&amp;ANOVA!C28&amp;")"</f>
         <v>61.72  (df = 3, 401)</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B10" s="32">
         <f>ANOVA!F27</f>
         <v>7.9203649667051561E-33</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B11" s="30">
         <f>ANOVA!B31</f>
         <v>0.31589325419476533</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="B12" s="28" t="str">
         <f>TEXT(ANOVA!C9,"0.00")&amp;" and "&amp;TEXT(ANOVA!C12,"0.00")</f>
         <v>3.99 and 5.51</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="B13" s="28" t="str">
         <f>TEXT(ANOVA!B38,"0.00")&amp;" (p = "&amp;TEXT(ANOVA!B41,"0.0E+00")&amp;")"</f>
         <v>80.89 (p = 6.2E-33)</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="B14" s="28" t="str">
         <f>TEXT(ANOVA!B47,"0.00")&amp;" (p = "&amp;TEXT(ANOVA!B49,"0.0E+00")&amp;")"</f>
         <v>129.79 (p = 6.0E-28)</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B15" s="30" t="str">
         <f>ANOVA!B32</f>
         <v>Reject H0: mean satisfaction differs across freshness levels</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2051,7 +2054,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="140" customWidth="1"/>
@@ -2059,57 +2062,62 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
-        <v>248</v>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="33" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -2129,161 +2137,161 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2298,46 +2306,46 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>67</v>
-      </c>
       <c r="M1" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -2384,7 +2392,7 @@
         <v>3</v>
       </c>
       <c r="P2" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -2431,7 +2439,7 @@
         <v>5</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -20183,83 +20191,83 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" s="10">
         <f>COUNT(Data!A2:A406)</f>
         <v>405</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTBLANK(Data!B2:N406)</f>
         <v>0</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B6" s="10">
         <f>SUMPRODUCT(--(COUNTIF(Data!A2:A406,Data!A2:A406)&gt;1))</f>
         <v>0</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B7" s="10">
         <f>COUNTIF(Data!B2:N406,"&lt;1")+COUNTIF(Data!B2:N406,"&gt;7")</f>
         <v>0</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B8" s="10">
         <f>SUMPRODUCT(--(Data!B2:N406&lt;&gt;INT(Data!B2:N406)))</f>
         <v>0</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -20281,46 +20289,46 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C4" s="10">
         <f>COUNT(Data!B$2:B$406)</f>
@@ -20349,10 +20357,10 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C5" s="10">
         <f>COUNT(Data!C$2:C$406)</f>
@@ -20381,10 +20389,10 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C6" s="10">
         <f>COUNT(Data!D$2:D$406)</f>
@@ -20413,10 +20421,10 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C7" s="10">
         <f>COUNT(Data!E$2:E$406)</f>
@@ -20445,10 +20453,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C8" s="10">
         <f>COUNT(Data!F$2:F$406)</f>
@@ -20477,10 +20485,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C9" s="10">
         <f>COUNT(Data!G$2:G$406)</f>
@@ -20509,10 +20517,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C10" s="10">
         <f>COUNT(Data!H$2:H$406)</f>
@@ -20541,10 +20549,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C11" s="10">
         <f>COUNT(Data!I$2:I$406)</f>
@@ -20573,10 +20581,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C12" s="10">
         <f>COUNT(Data!J$2:J$406)</f>
@@ -20605,10 +20613,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C13" s="10">
         <f>COUNT(Data!K$2:K$406)</f>
@@ -20637,10 +20645,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C14" s="10">
         <f>COUNT(Data!L$2:L$406)</f>
@@ -20669,10 +20677,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C15" s="10">
         <f>COUNT(Data!M$2:M$406)</f>
@@ -20701,10 +20709,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" s="10">
         <f>COUNT(Data!N$2:N$406)</f>
@@ -20748,17 +20756,17 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B3" s="10">
         <f>COUNT(Data!A2:A406)</f>
@@ -20767,7 +20775,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B4" s="14">
         <v>0.05</v>
@@ -20775,7 +20783,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B5" s="15">
         <f>B3-2</f>
@@ -20784,7 +20792,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B6" s="16">
         <f>_xlfn.T.INV.2T(B4,B5)</f>
@@ -20793,7 +20801,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B7" s="16">
         <f>B6/SQRT(B6^2+B5)</f>
@@ -20803,48 +20811,48 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="6"/>
       <c r="B9" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="I9" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="K9" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="L9" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="L9" s="6" t="s">
-        <v>67</v>
-      </c>
       <c r="M9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B10" s="17">
         <f>CORREL(Data!B$2:B$406,Data!B$2:B$406)</f>
@@ -20901,7 +20909,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B11" s="17">
         <f>CORREL(Data!C$2:C$406,Data!B$2:B$406)</f>
@@ -20958,7 +20966,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B12" s="17">
         <f>CORREL(Data!D$2:D$406,Data!B$2:B$406)</f>
@@ -21015,7 +21023,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B13" s="17">
         <f>CORREL(Data!E$2:E$406,Data!B$2:B$406)</f>
@@ -21072,7 +21080,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B14" s="17">
         <f>CORREL(Data!F$2:F$406,Data!B$2:B$406)</f>
@@ -21129,7 +21137,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B15" s="17">
         <f>CORREL(Data!G$2:G$406,Data!B$2:B$406)</f>
@@ -21186,7 +21194,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B16" s="17">
         <f>CORREL(Data!H$2:H$406,Data!B$2:B$406)</f>
@@ -21243,7 +21251,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B17" s="17">
         <f>CORREL(Data!I$2:I$406,Data!B$2:B$406)</f>
@@ -21300,7 +21308,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B18" s="17">
         <f>CORREL(Data!J$2:J$406,Data!B$2:B$406)</f>
@@ -21357,7 +21365,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B19" s="17">
         <f>CORREL(Data!K$2:K$406,Data!B$2:B$406)</f>
@@ -21414,7 +21422,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B20" s="17">
         <f>CORREL(Data!L$2:L$406,Data!B$2:B$406)</f>
@@ -21471,7 +21479,7 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B21" s="17">
         <f>CORREL(Data!M$2:M$406,Data!B$2:B$406)</f>
@@ -21528,7 +21536,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B22" s="17">
         <f>CORREL(Data!N$2:N$406,Data!B$2:B$406)</f>
@@ -21585,50 +21593,50 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="G25" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="J25" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C26" s="18">
         <f t="shared" ref="C26:C35" si="0">L10</f>
@@ -21669,10 +21677,10 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C27" s="18">
         <f t="shared" si="0"/>
@@ -21713,10 +21721,10 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C28" s="18">
         <f t="shared" si="0"/>
@@ -21757,10 +21765,10 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C29" s="18">
         <f t="shared" si="0"/>
@@ -21801,10 +21809,10 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C30" s="18">
         <f t="shared" si="0"/>
@@ -21845,10 +21853,10 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C31" s="18">
         <f t="shared" si="0"/>
@@ -21889,10 +21897,10 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C32" s="18">
         <f t="shared" si="0"/>
@@ -21933,10 +21941,10 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C33" s="18">
         <f t="shared" si="0"/>
@@ -21977,10 +21985,10 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C34" s="18">
         <f t="shared" si="0"/>
@@ -22021,10 +22029,10 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C35" s="18">
         <f t="shared" si="0"/>
@@ -22065,7 +22073,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C37" s="15">
         <f>COUNTIF(D26:D35,"&lt;"&amp;$B$4)+COUNTIF(G26:G35,"&lt;"&amp;$B$4)+COUNTIF(J26:J35,"&lt;"&amp;$B$4)</f>
@@ -22074,12 +22082,12 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>144</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -22113,25 +22121,25 @@
   <sheetData>
     <row r="1" spans="1:9" ht="51" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -22161,7 +22169,7 @@
         <v>112.5</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -22191,7 +22199,7 @@
         <v>112.5</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -32523,7 +32531,7 @@
         <v>5.5149700598802394</v>
       </c>
       <c r="E386" s="20">
-        <f t="shared" ref="E386:E449" si="25">(C386-D386)^2</f>
+        <f t="shared" ref="E386:E406" si="25">(C386-D386)^2</f>
         <v>0.23525404281257858</v>
       </c>
       <c r="F386" s="20">
@@ -33095,17 +33103,17 @@
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B4" s="22">
         <f>Correlation!B4</f>
@@ -33114,7 +33122,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B5" s="15">
         <f>COUNT(A9:A12)</f>
@@ -33123,34 +33131,34 @@
     </row>
     <row r="8" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -33319,7 +33327,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B13" s="15">
         <f>SUM(B9:B12)</f>
@@ -33332,7 +33340,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B15" s="17">
         <f>MAX(D9:D12)/MIN(D9:D12)</f>
@@ -33341,12 +33349,12 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B18" s="24">
         <f>AVERAGE('ANOVA Data'!F2:F406)</f>
@@ -33355,7 +33363,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B19" s="16">
         <f>SUMPRODUCT(B9:B12,(G9:G12-B18)^2)</f>
@@ -33364,7 +33372,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B20" s="24">
         <f>DEVSQ('ANOVA Data'!F2:F406)-B19</f>
@@ -33373,7 +33381,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B21" s="18">
         <f>(B19/(B5-1))/(B20/(B13-B5))</f>
@@ -33382,7 +33390,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B22" s="19">
         <f>_xlfn.F.DIST.RT(B21,B5-1,B13-B5)</f>
@@ -33391,7 +33399,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B23" s="9" t="str">
         <f>IF(B22&lt;B4,"No: variances differ (assumption violated)","Yes")</f>
@@ -33400,35 +33408,35 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="F26" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B27" s="16">
         <f>SUMPRODUCT(B9:B12,(C9:C12-C13)^2)</f>
@@ -33457,7 +33465,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B28" s="16">
         <f>SUM(H9:H12)</f>
@@ -33474,7 +33482,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B29" s="24">
         <f>DEVSQ('ANOVA Data'!C2:C406)</f>
@@ -33487,7 +33495,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B30" s="25">
         <f>B27+B28-B29</f>
@@ -33496,7 +33504,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B31" s="18">
         <f>B27/B29</f>
@@ -33505,7 +33513,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B32" s="9" t="str">
         <f>IF(F27&lt;B4,"Reject H0: mean satisfaction differs across freshness levels","Fail to reject H0")</f>
@@ -33514,12 +33522,12 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B35" s="16">
         <f>SUMPRODUCT(I9:I12,C9:C12)/SUM(I9:I12)</f>
@@ -33528,7 +33536,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B36" s="16">
         <f>SUMPRODUCT(I9:I12,(C9:C12-B35)^2)/(B5-1)</f>
@@ -33537,7 +33545,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B37" s="25">
         <f>SUM(J9:J12)</f>
@@ -33546,7 +33554,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B38" s="18">
         <f>B36/(1+2*(B5-2)/(B5^2-1)*B37)</f>
@@ -33555,7 +33563,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B39" s="15">
         <f>B5-1</f>
@@ -33564,7 +33572,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B40" s="17">
         <f>(B5^2-1)/(3*B37)</f>
@@ -33573,35 +33581,35 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B41" s="19">
         <f>_xlfn.F.DIST.RT(B38,B39,B40)</f>
         <v>6.1624459427165265E-33</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>193</v>
+        <v>247</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E44" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B45" s="18">
         <f>12/(B13*(B13+1))*SUMPRODUCT(F9:F12^2/B9:B12)-3*(B13+1)</f>
@@ -33621,7 +33629,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B46" s="16">
         <f>1-SUM(G45:G51)/(B13^3-B13)</f>
@@ -33641,7 +33649,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B47" s="18">
         <f>B45/B46</f>
@@ -33661,7 +33669,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B48" s="15">
         <f>B5-1</f>
@@ -33681,7 +33689,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B49" s="19">
         <f>_xlfn.CHISQ.DIST.RT(B47,B48)</f>
@@ -33727,29 +33735,29 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B54" s="17">
         <f>E27</f>
@@ -33770,7 +33778,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B55" s="17">
         <f>B38</f>
@@ -33791,7 +33799,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B56" s="17">
         <f>B47</f>
@@ -33812,7 +33820,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -33831,15 +33839,15 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="12:13" x14ac:dyDescent="0.25">
       <c r="L21" s="6" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="12:13" x14ac:dyDescent="0.25">
@@ -33944,7 +33952,7 @@
     </row>
     <row r="33" spans="12:12" x14ac:dyDescent="0.25">
       <c r="L33" s="8" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>